<commit_message>
Knockout stage round ready for deployment, results back up done
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08B58640-2A41-4BEB-9CFC-A1B2EC5B3E3F}"/>
+  <xr:revisionPtr revIDLastSave="180" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{099F8342-4399-4829-91B9-99049103DC9D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIFA World Cup 2026" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FIFA World Cup 2026'!$A$1:$D$105</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="427">
   <si>
     <t>Match</t>
   </si>
@@ -476,36 +476,18 @@
     <t>HRV GHA</t>
   </si>
   <si>
-    <t>Group A Runner-up vs Group B Runner-up</t>
-  </si>
-  <si>
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>Group E Winner vs Best 3rd (A/B/C/D/F)</t>
-  </si>
-  <si>
-    <t>Group F Winner vs Group C Runner-up</t>
-  </si>
-  <si>
-    <t>Group C Winner vs Group F Runner-up</t>
-  </si>
-  <si>
     <t>Group I Winner vs Best 3rd (C/D/F/G/H)</t>
   </si>
   <si>
     <t>Group E Runner-up vs Group I Runner-up</t>
   </si>
   <si>
-    <t>Group A Winner vs Best 3rd (C/E/F/H/I)</t>
-  </si>
-  <si>
     <t>Group L Winner vs Best 3rd (E/H/I/J/K)</t>
   </si>
   <si>
-    <t>Group D Winner vs Best 3rd (B/E/F/I/J)</t>
-  </si>
-  <si>
     <t>Group G Winner vs Best 3rd (A/E/H/I/J)</t>
   </si>
   <si>
@@ -515,12 +497,6 @@
     <t>Group H Winner vs Group J Runner-up</t>
   </si>
   <si>
-    <t>Group B Winner vs Best 3rd (E/F/G/I/J)</t>
-  </si>
-  <si>
-    <t>Group J Winner vs Group H Runner-up</t>
-  </si>
-  <si>
     <t>Group K Winner vs Best 3rd (D/E/I/J/L)</t>
   </si>
   <si>
@@ -1178,102 +1154,6 @@
     <t>Panama</t>
   </si>
   <si>
-    <t>Group A Runner-up</t>
-  </si>
-  <si>
-    <t>Group B Runner-up</t>
-  </si>
-  <si>
-    <t>Group E Winner</t>
-  </si>
-  <si>
-    <t>rd (A/B/C/D/F)</t>
-  </si>
-  <si>
-    <t>Group F Winner</t>
-  </si>
-  <si>
-    <t>up C Runner-up</t>
-  </si>
-  <si>
-    <t>Group C Winner</t>
-  </si>
-  <si>
-    <t>up F Runner-up</t>
-  </si>
-  <si>
-    <t>Group I Winner</t>
-  </si>
-  <si>
-    <t>rd (C/D/F/G/H)</t>
-  </si>
-  <si>
-    <t>Group E Runner-up</t>
-  </si>
-  <si>
-    <t>Group I Runner-up</t>
-  </si>
-  <si>
-    <t>Group A Winner</t>
-  </si>
-  <si>
-    <t>rd (C/E/F/H/I)</t>
-  </si>
-  <si>
-    <t>Group L Winner</t>
-  </si>
-  <si>
-    <t>rd (E/H/I/J/K)</t>
-  </si>
-  <si>
-    <t>Group D Winner</t>
-  </si>
-  <si>
-    <t>rd (B/E/F/I/J)</t>
-  </si>
-  <si>
-    <t>Group G Winner</t>
-  </si>
-  <si>
-    <t>rd (A/E/H/I/J)</t>
-  </si>
-  <si>
-    <t>Group K Runner-up</t>
-  </si>
-  <si>
-    <t>Group L Runner-up</t>
-  </si>
-  <si>
-    <t>Group H Winner</t>
-  </si>
-  <si>
-    <t>up J Runner-up</t>
-  </si>
-  <si>
-    <t>Group B Winner</t>
-  </si>
-  <si>
-    <t>rd (E/F/G/I/J)</t>
-  </si>
-  <si>
-    <t>Group J Winner</t>
-  </si>
-  <si>
-    <t>up H Runner-up</t>
-  </si>
-  <si>
-    <t>Group K Winner</t>
-  </si>
-  <si>
-    <t>rd (D/E/I/J/L)</t>
-  </si>
-  <si>
-    <t>Group D Runner-up</t>
-  </si>
-  <si>
-    <t>Group G Runner-up</t>
-  </si>
-  <si>
     <t>R32 Match 2 Winner</t>
   </si>
   <si>
@@ -1379,75 +1259,9 @@
     <t>Round of 32</t>
   </si>
   <si>
-    <t>Round of 33</t>
-  </si>
-  <si>
-    <t>Round of 34</t>
-  </si>
-  <si>
-    <t>Round of 35</t>
-  </si>
-  <si>
-    <t>Round of 36</t>
-  </si>
-  <si>
-    <t>Round of 37</t>
-  </si>
-  <si>
-    <t>Round of 38</t>
-  </si>
-  <si>
-    <t>Round of 39</t>
-  </si>
-  <si>
-    <t>Round of 40</t>
-  </si>
-  <si>
-    <t>Round of 41</t>
-  </si>
-  <si>
-    <t>Round of 42</t>
-  </si>
-  <si>
-    <t>Round of 43</t>
-  </si>
-  <si>
-    <t>Round of 44</t>
-  </si>
-  <si>
-    <t>Round of 45</t>
-  </si>
-  <si>
-    <t>Round of 46</t>
-  </si>
-  <si>
-    <t>Round of 47</t>
-  </si>
-  <si>
     <t>Round of 16</t>
   </si>
   <si>
-    <t>Round of 17</t>
-  </si>
-  <si>
-    <t>Round of 18</t>
-  </si>
-  <si>
-    <t>Round of 19</t>
-  </si>
-  <si>
-    <t>Round of 20</t>
-  </si>
-  <si>
-    <t>Round of 21</t>
-  </si>
-  <si>
-    <t>Round of 22</t>
-  </si>
-  <si>
-    <t>Round of 23</t>
-  </si>
-  <si>
     <t>Quarterfinal</t>
   </si>
   <si>
@@ -1455,6 +1269,54 @@
   </si>
   <si>
     <t>3rd Place</t>
+  </si>
+  <si>
+    <t>South Africa vs Canada</t>
+  </si>
+  <si>
+    <t>Germany vs Best 3rd (A/B/C/D/F)</t>
+  </si>
+  <si>
+    <t>Group F Winner vs Morocco</t>
+  </si>
+  <si>
+    <t>Brazil vs Group F Runner-up</t>
+  </si>
+  <si>
+    <t>Mexico vs Best 3rd (C/E/F/H/I)</t>
+  </si>
+  <si>
+    <t>USA vs Best 3rd (B/E/F/I/J)</t>
+  </si>
+  <si>
+    <t>Switzerland vs Best 3rd (E/F/G/I/J)</t>
+  </si>
+  <si>
+    <t>Argentina vs Group H Runner-up</t>
+  </si>
+  <si>
+    <t>ZAF CAN</t>
+  </si>
+  <si>
+    <t>DEU TBD</t>
+  </si>
+  <si>
+    <t>TBD MAR</t>
+  </si>
+  <si>
+    <t>BRA TBD</t>
+  </si>
+  <si>
+    <t>MEX TBD</t>
+  </si>
+  <si>
+    <t>USA TBD</t>
+  </si>
+  <si>
+    <t>CHE TBD</t>
+  </si>
+  <si>
+    <t>ARG TBD</t>
   </si>
 </sst>
 </file>
@@ -2095,22 +1957,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2118,22 +1980,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2141,22 +2003,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="F3" s="36" t="s">
         <v>276</v>
       </c>
-      <c r="F3" s="36" t="s">
-        <v>284</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2164,22 +2026,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2187,22 +2049,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2210,22 +2072,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2233,22 +2095,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2256,22 +2118,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2279,22 +2141,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2302,22 +2164,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2325,22 +2187,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2348,22 +2210,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2371,22 +2233,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2394,22 +2256,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2417,22 +2279,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2440,22 +2302,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2463,22 +2325,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2486,22 +2348,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2509,22 +2371,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2532,22 +2394,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2555,22 +2417,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2578,22 +2440,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2601,22 +2463,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2624,22 +2486,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2647,22 +2509,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2670,22 +2532,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2693,22 +2555,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>444</v>
+        <v>404</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>445</v>
+        <v>405</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2716,22 +2578,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>444</v>
+        <v>404</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2739,22 +2601,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2762,22 +2624,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2785,22 +2647,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>444</v>
+        <v>404</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2808,22 +2670,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2831,22 +2693,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2854,22 +2716,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2877,22 +2739,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2900,22 +2762,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2923,22 +2785,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2946,22 +2808,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2969,22 +2831,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2992,22 +2854,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3015,22 +2877,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3038,22 +2900,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3061,22 +2923,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3084,22 +2946,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3107,22 +2969,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3130,22 +2992,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3153,22 +3015,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3176,22 +3038,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3199,22 +3061,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3222,22 +3084,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3245,22 +3107,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="C51" s="18" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3268,22 +3130,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="C52" s="18" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3291,22 +3153,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3314,22 +3176,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3337,22 +3199,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3360,22 +3222,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3383,22 +3245,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3406,22 +3268,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3429,22 +3291,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3452,22 +3314,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3475,22 +3337,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3498,22 +3360,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3521,22 +3383,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3544,22 +3406,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3567,22 +3429,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3590,22 +3452,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3613,22 +3475,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="C67" s="22" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3636,22 +3498,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="C68" s="24" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3659,22 +3521,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="C69" s="24" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3682,22 +3544,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3705,22 +3567,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3728,22 +3590,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3751,758 +3613,712 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="C73" s="24" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
-        <v>146</v>
+        <v>411</v>
       </c>
       <c r="B74" s="26" t="s">
-        <v>380</v>
+        <v>328</v>
       </c>
       <c r="C74" s="26" t="s">
-        <v>381</v>
+        <v>329</v>
       </c>
       <c r="D74" s="27" t="s">
-        <v>147</v>
+        <v>419</v>
       </c>
       <c r="E74" s="48" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>446</v>
+        <v>406</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>148</v>
+        <v>412</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>382</v>
-      </c>
-      <c r="C75" s="26" t="s">
-        <v>383</v>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="C75" s="26"/>
       <c r="D75" s="27" t="s">
-        <v>147</v>
+        <v>420</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>447</v>
+        <v>406</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="B76" s="26" t="s">
-        <v>384</v>
-      </c>
+        <v>413</v>
+      </c>
+      <c r="B76" s="26"/>
       <c r="C76" s="26" t="s">
-        <v>385</v>
+        <v>336</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>147</v>
+        <v>421</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>448</v>
+        <v>406</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>150</v>
+        <v>414</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>386</v>
-      </c>
-      <c r="C77" s="26" t="s">
-        <v>387</v>
-      </c>
+        <v>333</v>
+      </c>
+      <c r="C77" s="26"/>
       <c r="D77" s="27" t="s">
-        <v>147</v>
+        <v>422</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>449</v>
+        <v>406</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="B78" s="26" t="s">
-        <v>388</v>
-      </c>
-      <c r="C78" s="26" t="s">
-        <v>389</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
       <c r="D78" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>450</v>
+        <v>406</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="B79" s="26" t="s">
-        <v>390</v>
-      </c>
-      <c r="C79" s="26" t="s">
-        <v>391</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
       <c r="D79" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E79" s="48" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>451</v>
+        <v>406</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>153</v>
+        <v>415</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>392</v>
-      </c>
-      <c r="C80" s="26" t="s">
-        <v>393</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="C80" s="26"/>
       <c r="D80" s="27" t="s">
-        <v>147</v>
+        <v>423</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>452</v>
+        <v>406</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B81" s="26" t="s">
-        <v>394</v>
-      </c>
-      <c r="C81" s="26" t="s">
-        <v>395</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="B81" s="26"/>
+      <c r="C81" s="26"/>
       <c r="D81" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>453</v>
+        <v>406</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>155</v>
+        <v>416</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>396</v>
-      </c>
-      <c r="C82" s="26" t="s">
-        <v>397</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="C82" s="26"/>
       <c r="D82" s="27" t="s">
-        <v>147</v>
+        <v>424</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>454</v>
+        <v>406</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="B83" s="26" t="s">
-        <v>398</v>
-      </c>
-      <c r="C83" s="26" t="s">
-        <v>399</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="B83" s="26"/>
+      <c r="C83" s="26"/>
       <c r="D83" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>455</v>
+        <v>406</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="B84" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="C84" s="26" t="s">
-        <v>401</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="B84" s="26"/>
+      <c r="C84" s="26"/>
       <c r="D84" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>456</v>
+        <v>406</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="B85" s="26" t="s">
-        <v>402</v>
-      </c>
-      <c r="C85" s="26" t="s">
-        <v>403</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="B85" s="26"/>
+      <c r="C85" s="26"/>
       <c r="D85" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>457</v>
+        <v>406</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>159</v>
+        <v>417</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="C86" s="26" t="s">
-        <v>405</v>
-      </c>
+        <v>331</v>
+      </c>
+      <c r="C86" s="26"/>
       <c r="D86" s="27" t="s">
-        <v>147</v>
+        <v>425</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>458</v>
+        <v>406</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>160</v>
+        <v>418</v>
       </c>
       <c r="B87" s="26" t="s">
+        <v>360</v>
+      </c>
+      <c r="C87" s="26"/>
+      <c r="D87" s="27" t="s">
+        <v>426</v>
+      </c>
+      <c r="E87" s="48" t="s">
+        <v>248</v>
+      </c>
+      <c r="F87" s="48" t="s">
+        <v>317</v>
+      </c>
+      <c r="G87" s="27" t="s">
         <v>406</v>
-      </c>
-      <c r="C87" s="26" t="s">
-        <v>407</v>
-      </c>
-      <c r="D87" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="E87" s="48" t="s">
-        <v>256</v>
-      </c>
-      <c r="F87" s="48" t="s">
-        <v>325</v>
-      </c>
-      <c r="G87" s="27" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="B88" s="26" t="s">
-        <v>408</v>
-      </c>
-      <c r="C88" s="26" t="s">
-        <v>409</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="B88" s="26"/>
+      <c r="C88" s="26"/>
       <c r="D88" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>460</v>
+        <v>406</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="B89" s="26" t="s">
-        <v>410</v>
-      </c>
-      <c r="C89" s="26" t="s">
-        <v>411</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="B89" s="26"/>
+      <c r="C89" s="26"/>
       <c r="D89" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>461</v>
+        <v>406</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>412</v>
+        <v>372</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>413</v>
+        <v>373</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>462</v>
+        <v>407</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>414</v>
+        <v>374</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>415</v>
+        <v>375</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>463</v>
+        <v>407</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>416</v>
+        <v>376</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>417</v>
+        <v>377</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>464</v>
+        <v>407</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>418</v>
+        <v>378</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>419</v>
+        <v>379</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>465</v>
+        <v>407</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>420</v>
+        <v>380</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>421</v>
+        <v>381</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>466</v>
+        <v>407</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>422</v>
+        <v>382</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>423</v>
+        <v>383</v>
       </c>
       <c r="D95" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>467</v>
+        <v>407</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>424</v>
+        <v>384</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>425</v>
+        <v>385</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>468</v>
+        <v>407</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>426</v>
+        <v>386</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>427</v>
+        <v>387</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>469</v>
+        <v>407</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>428</v>
+        <v>388</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>429</v>
+        <v>389</v>
       </c>
       <c r="D98" s="31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>470</v>
+        <v>408</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>430</v>
+        <v>390</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>431</v>
+        <v>391</v>
       </c>
       <c r="D99" s="31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>470</v>
+        <v>408</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>432</v>
+        <v>392</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>433</v>
+        <v>393</v>
       </c>
       <c r="D100" s="31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>470</v>
+        <v>408</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>434</v>
+        <v>394</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>435</v>
+        <v>395</v>
       </c>
       <c r="D101" s="31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>470</v>
+        <v>408</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="B102" s="32" t="s">
-        <v>436</v>
+        <v>396</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>437</v>
+        <v>397</v>
       </c>
       <c r="D102" s="33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>471</v>
+        <v>409</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>438</v>
+        <v>398</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>439</v>
+        <v>399</v>
       </c>
       <c r="D103" s="33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>471</v>
+        <v>409</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B104" s="34" t="s">
-        <v>440</v>
+        <v>400</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>441</v>
+        <v>401</v>
       </c>
       <c r="D104" s="35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>472</v>
+        <v>410</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>442</v>
+        <v>402</v>
       </c>
       <c r="C105" s="26" t="s">
-        <v>443</v>
+        <v>403</v>
       </c>
       <c r="D105" s="27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
knockout stage 1st commit. miss draw + penalty and goalscorer
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{601AE739-FDCD-420E-AF9E-14D320C706D4}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8641F9B3-615B-4E99-BE06-9467D6DC15F6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="434">
   <si>
     <t>Match</t>
   </si>
@@ -482,9 +482,6 @@
     <t>R32 Match 2 Winner vs R32 Match 5 Winner</t>
   </si>
   <si>
-    <t>R32 Match 1 Winner vs R32 Match 3 Winner</t>
-  </si>
-  <si>
     <t>R32 Match 4 Winner vs R32 Match 6 Winner</t>
   </si>
   <si>
@@ -1136,9 +1133,6 @@
     <t>R32 Match 5 Winner</t>
   </si>
   <si>
-    <t>R32 Match 1 Winner</t>
-  </si>
-  <si>
     <t>R32 Match 3 Winner</t>
   </si>
   <si>
@@ -1341,6 +1335,9 @@
   </si>
   <si>
     <t>COL GHA</t>
+  </si>
+  <si>
+    <t>Canada vs R32 Match 3 Winner</t>
   </si>
 </sst>
 </file>
@@ -1981,22 +1978,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2004,22 +2001,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2027,22 +2024,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>318</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>319</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2050,22 +2047,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>320</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2073,22 +2070,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>318</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2096,22 +2093,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2119,22 +2116,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2142,22 +2139,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2165,22 +2162,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>323</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2188,22 +2185,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>324</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2211,22 +2208,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>321</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>322</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2234,22 +2231,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2257,22 +2254,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2280,22 +2277,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2303,22 +2300,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>327</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2326,22 +2323,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>328</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2349,22 +2346,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2372,22 +2369,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2395,22 +2392,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2418,22 +2415,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2441,22 +2438,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>330</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>331</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2464,22 +2461,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>331</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>332</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2487,22 +2484,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>329</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2510,22 +2507,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2533,22 +2530,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2556,22 +2553,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>333</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>334</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2579,22 +2576,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2602,22 +2599,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2625,22 +2622,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2648,22 +2645,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2671,22 +2668,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2694,22 +2691,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2717,22 +2714,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>337</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>338</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2740,22 +2737,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>336</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>337</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2763,22 +2760,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>338</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>339</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2786,22 +2783,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2809,22 +2806,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2832,22 +2829,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2855,22 +2852,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>341</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>342</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2878,22 +2875,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>340</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>341</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2901,22 +2898,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>342</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>343</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2924,22 +2921,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2947,22 +2944,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2970,22 +2967,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2993,22 +2990,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>345</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>346</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3016,22 +3013,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>344</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>345</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3039,22 +3036,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>346</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>347</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3062,22 +3059,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3085,22 +3082,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3108,22 +3105,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3131,22 +3128,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>349</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>350</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3154,22 +3151,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>348</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>349</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3177,22 +3174,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>350</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>351</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3200,22 +3197,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3223,22 +3220,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3246,22 +3243,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3269,22 +3266,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>353</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>354</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3292,22 +3289,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>352</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>353</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3315,22 +3312,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>353</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>354</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>355</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3338,22 +3335,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3361,22 +3358,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3384,22 +3381,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>356</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>357</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3407,22 +3404,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>357</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>358</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>359</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3430,22 +3427,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3453,22 +3450,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3476,22 +3473,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3499,22 +3496,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>357</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>358</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3522,22 +3519,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>359</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>360</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>361</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3545,22 +3542,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>361</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>362</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>363</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3568,22 +3565,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3591,22 +3588,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3614,22 +3611,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3637,390 +3634,390 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>360</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>361</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>362</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B74" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="C74" s="26" t="s">
         <v>320</v>
       </c>
-      <c r="C74" s="26" t="s">
-        <v>321</v>
-      </c>
       <c r="D74" s="27" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E74" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B79" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="C79" s="26" t="s">
+        <v>349</v>
+      </c>
+      <c r="D79" s="27" t="s">
+        <v>416</v>
+      </c>
+      <c r="E79" s="48" t="s">
+        <v>231</v>
+      </c>
+      <c r="F79" s="48" t="s">
+        <v>308</v>
+      </c>
+      <c r="G79" s="27" t="s">
         <v>396</v>
-      </c>
-      <c r="C79" s="26" t="s">
-        <v>350</v>
-      </c>
-      <c r="D79" s="27" t="s">
-        <v>418</v>
-      </c>
-      <c r="E79" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="F79" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="G79" s="27" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -4028,367 +4025,367 @@
         <v>147</v>
       </c>
       <c r="B90" s="28" t="s">
+        <v>363</v>
+      </c>
+      <c r="C90" s="28" t="s">
         <v>364</v>
-      </c>
-      <c r="C90" s="28" t="s">
-        <v>365</v>
       </c>
       <c r="D90" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>148</v>
+        <v>433</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>366</v>
+        <v>320</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D91" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D92" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D93" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D94" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D95" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D96" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D97" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D98" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D99" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D100" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D101" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B102" s="32" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D102" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D103" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B104" s="34" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C105" s="26" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D105" s="27" t="s">
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
scorer works for single goal
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8641F9B3-615B-4E99-BE06-9467D6DC15F6}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAE77228-A57A-48DE-A4BB-549B54395AAE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="435">
   <si>
     <t>Match</t>
   </si>
@@ -482,9 +482,6 @@
     <t>R32 Match 2 Winner vs R32 Match 5 Winner</t>
   </si>
   <si>
-    <t>R32 Match 4 Winner vs R32 Match 6 Winner</t>
-  </si>
-  <si>
     <t>R32 Match 7 Winner vs R32 Match 8 Winner</t>
   </si>
   <si>
@@ -1136,9 +1133,6 @@
     <t>R32 Match 3 Winner</t>
   </si>
   <si>
-    <t>R32 Match 4 Winner</t>
-  </si>
-  <si>
     <t>R32 Match 6 Winner</t>
   </si>
   <si>
@@ -1338,6 +1332,15 @@
   </si>
   <si>
     <t>Canada vs R32 Match 3 Winner</t>
+  </si>
+  <si>
+    <t>Brazil vs R32 Match 6 Winner</t>
+  </si>
+  <si>
+    <t>BRA TBD</t>
+  </si>
+  <si>
+    <t>CAN TBD</t>
   </si>
 </sst>
 </file>
@@ -1978,22 +1981,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>314</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>315</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2001,22 +2004,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2024,22 +2027,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>318</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2047,22 +2050,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>318</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>319</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2070,22 +2073,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>317</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2093,22 +2096,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2116,22 +2119,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2139,22 +2142,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2162,22 +2165,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>321</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>322</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2185,22 +2188,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>323</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2208,22 +2211,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>320</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>321</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2231,22 +2234,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2254,22 +2257,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2277,22 +2280,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2300,22 +2303,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2323,22 +2326,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>327</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2346,22 +2349,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>324</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>325</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2369,22 +2372,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2392,22 +2395,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2415,22 +2418,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2438,22 +2441,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>329</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2461,22 +2464,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>330</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>331</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2484,22 +2487,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>328</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>329</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2507,22 +2510,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2530,22 +2533,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2553,22 +2556,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>332</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>333</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2576,22 +2579,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2599,22 +2602,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2622,22 +2625,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2645,22 +2648,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2668,22 +2671,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2691,22 +2694,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2714,22 +2717,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>336</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>337</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2737,22 +2740,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>335</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>336</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2760,22 +2763,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>337</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>338</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2783,22 +2786,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2806,22 +2809,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2829,22 +2832,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2852,22 +2855,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>340</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>341</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2875,22 +2878,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>339</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>340</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2898,22 +2901,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>341</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>342</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2921,22 +2924,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2944,22 +2947,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2967,22 +2970,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2990,22 +2993,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>344</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>345</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3013,22 +3016,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>343</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>344</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3036,22 +3039,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>345</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>346</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3059,22 +3062,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3082,22 +3085,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3105,22 +3108,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3128,22 +3131,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>348</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>349</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3151,22 +3154,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>347</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>348</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3174,22 +3177,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>349</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>350</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3197,22 +3200,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3220,22 +3223,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3243,22 +3246,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3266,22 +3269,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>352</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>353</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3289,22 +3292,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>351</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>352</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3312,22 +3315,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>353</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>354</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3335,22 +3338,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3358,22 +3361,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3381,22 +3384,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>354</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>355</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>356</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3404,22 +3407,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>357</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>358</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3427,22 +3430,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3450,22 +3453,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3473,22 +3476,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3496,22 +3499,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>356</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>357</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3519,22 +3522,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>358</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>359</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>360</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3542,22 +3545,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>360</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>361</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>362</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3565,22 +3568,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3588,22 +3591,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3611,22 +3614,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3634,390 +3637,390 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>359</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>360</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>361</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B74" s="26" t="s">
+        <v>318</v>
+      </c>
+      <c r="C74" s="26" t="s">
         <v>319</v>
       </c>
-      <c r="C74" s="26" t="s">
-        <v>320</v>
-      </c>
       <c r="D74" s="27" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E74" s="48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B79" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="C79" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="D79" s="27" t="s">
+        <v>414</v>
+      </c>
+      <c r="E79" s="48" t="s">
+        <v>230</v>
+      </c>
+      <c r="F79" s="48" t="s">
+        <v>307</v>
+      </c>
+      <c r="G79" s="27" t="s">
         <v>394</v>
-      </c>
-      <c r="C79" s="26" t="s">
-        <v>349</v>
-      </c>
-      <c r="D79" s="27" t="s">
-        <v>416</v>
-      </c>
-      <c r="E79" s="48" t="s">
-        <v>231</v>
-      </c>
-      <c r="F79" s="48" t="s">
-        <v>308</v>
-      </c>
-      <c r="G79" s="27" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -4025,367 +4028,367 @@
         <v>147</v>
       </c>
       <c r="B90" s="28" t="s">
+        <v>362</v>
+      </c>
+      <c r="C90" s="28" t="s">
         <v>363</v>
-      </c>
-      <c r="C90" s="28" t="s">
-        <v>364</v>
       </c>
       <c r="D90" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>146</v>
+        <v>434</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>148</v>
+        <v>432</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>366</v>
+        <v>323</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>146</v>
+        <v>433</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D93" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D94" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D95" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D96" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D97" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D98" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D99" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D100" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D101" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B102" s="32" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D102" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D103" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B104" s="34" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C105" s="26" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D105" s="27" t="s">
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Double scorer + date glitch solved
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="224" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81BAC917-BD05-4738-82A0-A31BC17FBC43}"/>
+  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9593630-3092-4AE9-9261-D040FD3D8128}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIFA World Cup 2026" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="422">
   <si>
     <t>Match</t>
   </si>
@@ -479,9 +479,6 @@
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>R32 Match 7 Winner vs R32 Match 8 Winner</t>
-  </si>
-  <si>
     <t>R32 Match 11 Winner vs R32 Match 12 Winner</t>
   </si>
   <si>
@@ -1286,15 +1283,9 @@
     <t>COL GHA</t>
   </si>
   <si>
-    <t>Brazil vs R32 Match 6 Winner</t>
-  </si>
-  <si>
     <t>BRA TBD</t>
   </si>
   <si>
-    <t>Paraguay vs R32 Match 5 Winner</t>
-  </si>
-  <si>
     <t>PRY TBD</t>
   </si>
   <si>
@@ -1302,6 +1293,15 @@
   </si>
   <si>
     <t>CAN MAR</t>
+  </si>
+  <si>
+    <t>Paraguay vs France</t>
+  </si>
+  <si>
+    <t>Brazil vs Norway</t>
+  </si>
+  <si>
+    <t>Mexico vs R32 Match 8 Winner</t>
   </si>
 </sst>
 </file>
@@ -1942,22 +1942,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1965,22 +1965,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1988,22 +1988,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>316</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2011,22 +2011,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>317</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2034,22 +2034,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>315</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2057,22 +2057,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2080,22 +2080,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2103,22 +2103,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2126,22 +2126,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2149,22 +2149,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>320</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>321</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2172,22 +2172,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>318</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>319</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2195,22 +2195,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2218,22 +2218,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2241,22 +2241,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2264,22 +2264,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>323</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>324</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2287,22 +2287,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>324</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>325</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2310,22 +2310,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>322</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>323</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2333,22 +2333,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2356,22 +2356,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2379,22 +2379,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2402,22 +2402,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>327</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>328</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2425,22 +2425,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>328</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>329</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2448,22 +2448,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>326</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>327</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2471,22 +2471,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2494,22 +2494,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2517,22 +2517,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>330</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>331</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2540,22 +2540,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2563,22 +2563,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2586,22 +2586,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2609,22 +2609,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2632,22 +2632,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2655,22 +2655,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2678,22 +2678,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>334</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>335</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2701,22 +2701,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>333</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>334</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2724,22 +2724,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>335</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>336</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2747,22 +2747,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2770,22 +2770,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2793,22 +2793,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2816,22 +2816,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>338</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>339</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2839,22 +2839,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>337</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>338</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2862,22 +2862,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>339</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>340</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2885,22 +2885,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2908,22 +2908,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2931,22 +2931,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2954,22 +2954,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>342</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>343</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2977,22 +2977,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>341</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>342</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3000,22 +3000,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>343</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>344</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3023,22 +3023,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3046,22 +3046,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3069,22 +3069,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3092,22 +3092,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>346</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>347</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3115,22 +3115,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>345</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>346</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3138,22 +3138,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>347</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>348</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3161,22 +3161,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3184,22 +3184,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3207,22 +3207,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3230,22 +3230,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>349</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>350</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>351</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3253,22 +3253,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>349</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>350</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3276,22 +3276,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>351</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>352</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3299,22 +3299,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3322,22 +3322,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3345,22 +3345,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>352</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>353</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>354</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3368,22 +3368,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>354</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>355</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>356</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3391,22 +3391,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3414,22 +3414,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3437,22 +3437,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3460,22 +3460,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>354</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>355</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3483,22 +3483,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>356</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>357</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>358</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3506,22 +3506,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>358</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>359</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>360</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3529,22 +3529,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3552,22 +3552,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3575,22 +3575,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3598,479 +3598,485 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>357</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>358</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>359</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
+        <v>383</v>
+      </c>
+      <c r="B74" s="26" t="s">
+        <v>316</v>
+      </c>
+      <c r="C74" s="26" t="s">
+        <v>317</v>
+      </c>
+      <c r="D74" s="27" t="s">
         <v>384</v>
       </c>
-      <c r="B74" s="26" t="s">
-        <v>317</v>
-      </c>
-      <c r="C74" s="26" t="s">
-        <v>318</v>
-      </c>
-      <c r="D74" s="27" t="s">
-        <v>385</v>
-      </c>
       <c r="E74" s="48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C79" s="26" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D79" s="27" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E79" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>329</v>
-      </c>
-      <c r="C90" s="28"/>
+        <v>328</v>
+      </c>
+      <c r="C90" s="28" t="s">
+        <v>344</v>
+      </c>
       <c r="D90" s="29" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>322</v>
-      </c>
-      <c r="C92" s="28"/>
+        <v>321</v>
+      </c>
+      <c r="C92" s="28" t="s">
+        <v>346</v>
+      </c>
       <c r="D92" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="B93" s="28"/>
+        <v>421</v>
+      </c>
+      <c r="B93" s="28" t="s">
+        <v>313</v>
+      </c>
       <c r="C93" s="28"/>
       <c r="D93" s="29" t="s">
         <v>146</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B94" s="28"/>
       <c r="C94" s="28"/>
@@ -4078,18 +4084,18 @@
         <v>146</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B95" s="28"/>
       <c r="C95" s="28"/>
@@ -4097,18 +4103,18 @@
         <v>146</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B96" s="28"/>
       <c r="C96" s="28"/>
@@ -4116,18 +4122,18 @@
         <v>146</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B97" s="28"/>
       <c r="C97" s="28"/>
@@ -4135,197 +4141,197 @@
         <v>146</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B98" s="30" t="s">
+        <v>360</v>
+      </c>
+      <c r="C98" s="30" t="s">
         <v>361</v>
-      </c>
-      <c r="C98" s="30" t="s">
-        <v>362</v>
       </c>
       <c r="D98" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B99" s="30" t="s">
+        <v>362</v>
+      </c>
+      <c r="C99" s="30" t="s">
         <v>363</v>
-      </c>
-      <c r="C99" s="30" t="s">
-        <v>364</v>
       </c>
       <c r="D99" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B100" s="30" t="s">
+        <v>364</v>
+      </c>
+      <c r="C100" s="30" t="s">
         <v>365</v>
-      </c>
-      <c r="C100" s="30" t="s">
-        <v>366</v>
       </c>
       <c r="D100" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B101" s="30" t="s">
+        <v>366</v>
+      </c>
+      <c r="C101" s="30" t="s">
         <v>367</v>
-      </c>
-      <c r="C101" s="30" t="s">
-        <v>368</v>
       </c>
       <c r="D101" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B102" s="32" t="s">
+        <v>368</v>
+      </c>
+      <c r="C102" s="32" t="s">
         <v>369</v>
-      </c>
-      <c r="C102" s="32" t="s">
-        <v>370</v>
       </c>
       <c r="D102" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B103" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="C103" s="32" t="s">
         <v>371</v>
-      </c>
-      <c r="C103" s="32" t="s">
-        <v>372</v>
       </c>
       <c r="D103" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B104" s="34" t="s">
+        <v>372</v>
+      </c>
+      <c r="C104" s="34" t="s">
         <v>373</v>
-      </c>
-      <c r="C104" s="34" t="s">
-        <v>374</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B105" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="C105" s="26" t="s">
         <v>375</v>
-      </c>
-      <c r="C105" s="26" t="s">
-        <v>376</v>
       </c>
       <c r="D105" s="27" t="s">
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit july 04. round of 16 form loaded
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82144695-7534-423B-8F23-C0E9A7491753}"/>
+  <xr:revisionPtr revIDLastSave="253" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA247424-ECCB-4175-8CF7-412282A3F78A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="427">
   <si>
     <t>Match</t>
   </si>
@@ -479,12 +479,6 @@
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>R32 Match 14 Winner vs R32 Match 16 Winner</t>
-  </si>
-  <si>
-    <t>R32 Match 13 Winner vs R32 Match 15 Winner</t>
-  </si>
-  <si>
     <t>R16 Match 1 Winner vs R16 Match 2 Winner</t>
   </si>
   <si>
@@ -1277,12 +1271,6 @@
     <t>COL GHA</t>
   </si>
   <si>
-    <t>BRA TBD</t>
-  </si>
-  <si>
-    <t>PRY TBD</t>
-  </si>
-  <si>
     <t>Canada vs Morocco</t>
   </si>
   <si>
@@ -1311,6 +1299,24 @@
   </si>
   <si>
     <t>PRT ESP</t>
+  </si>
+  <si>
+    <t>PRY FRA</t>
+  </si>
+  <si>
+    <t>BRA NOR</t>
+  </si>
+  <si>
+    <t>Argentina vs Egypt</t>
+  </si>
+  <si>
+    <t>Switzerland vs Colombia</t>
+  </si>
+  <si>
+    <t>ARG EGY</t>
+  </si>
+  <si>
+    <t>CHE COL</t>
   </si>
 </sst>
 </file>
@@ -1951,22 +1957,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1974,22 +1980,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1997,22 +2003,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2020,22 +2026,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2043,22 +2049,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2066,22 +2072,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2089,22 +2095,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2112,22 +2118,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2135,22 +2141,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2158,22 +2164,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2181,22 +2187,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2204,22 +2210,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2227,22 +2233,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2250,22 +2256,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2273,22 +2279,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2296,22 +2302,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2319,22 +2325,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2342,22 +2348,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2365,22 +2371,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2388,22 +2394,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2411,22 +2417,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
+        <v>258</v>
+      </c>
+      <c r="F21" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="F21" s="36" t="s">
-        <v>262</v>
-      </c>
       <c r="G21" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2434,22 +2440,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2457,22 +2463,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2480,22 +2486,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2503,22 +2509,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2526,22 +2532,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2549,22 +2555,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2572,22 +2578,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2595,22 +2601,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2618,22 +2624,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2641,22 +2647,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2664,22 +2670,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2687,22 +2693,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2710,22 +2716,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2733,22 +2739,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2756,22 +2762,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2779,22 +2785,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2802,22 +2808,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2825,22 +2831,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2848,22 +2854,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2871,22 +2877,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2894,22 +2900,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2917,22 +2923,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2940,22 +2946,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2963,22 +2969,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2986,22 +2992,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3009,22 +3015,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3032,22 +3038,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3055,22 +3061,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3078,22 +3084,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3101,22 +3107,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C51" s="18" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3124,22 +3130,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C52" s="18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3147,22 +3153,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3170,22 +3176,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3193,22 +3199,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3216,22 +3222,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3239,22 +3245,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3262,22 +3268,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3285,22 +3291,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3308,22 +3314,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3331,22 +3337,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3354,22 +3360,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3377,22 +3383,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3400,22 +3406,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
+        <v>348</v>
+      </c>
+      <c r="C64" s="22" t="s">
         <v>350</v>
-      </c>
-      <c r="C64" s="22" t="s">
-        <v>352</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3423,22 +3429,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3446,22 +3452,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3469,22 +3475,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C67" s="22" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3492,22 +3498,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C68" s="24" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3515,22 +3521,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C69" s="24" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3538,22 +3544,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
+        <v>352</v>
+      </c>
+      <c r="C70" s="24" t="s">
         <v>354</v>
-      </c>
-      <c r="C70" s="24" t="s">
-        <v>356</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3561,22 +3567,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3584,22 +3590,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3607,750 +3613,758 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C73" s="24" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B74" s="26" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C74" s="26" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D74" s="27" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E74" s="48" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B79" s="26" t="s">
+        <v>372</v>
+      </c>
+      <c r="C79" s="26" t="s">
+        <v>342</v>
+      </c>
+      <c r="D79" s="27" t="s">
+        <v>394</v>
+      </c>
+      <c r="E79" s="48" t="s">
+        <v>224</v>
+      </c>
+      <c r="F79" s="48" t="s">
+        <v>301</v>
+      </c>
+      <c r="G79" s="27" t="s">
         <v>374</v>
-      </c>
-      <c r="C79" s="26" t="s">
-        <v>344</v>
-      </c>
-      <c r="D79" s="27" t="s">
-        <v>396</v>
-      </c>
-      <c r="E79" s="48" t="s">
-        <v>226</v>
-      </c>
-      <c r="F79" s="48" t="s">
-        <v>303</v>
-      </c>
-      <c r="G79" s="27" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>413</v>
+        <v>422</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D95" s="29" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="B96" s="28"/>
-      <c r="C96" s="28"/>
+        <v>423</v>
+      </c>
+      <c r="B96" s="28" t="s">
+        <v>344</v>
+      </c>
+      <c r="C96" s="28" t="s">
+        <v>335</v>
+      </c>
       <c r="D96" s="29" t="s">
-        <v>146</v>
+        <v>425</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="B97" s="28"/>
-      <c r="C97" s="28"/>
+        <v>424</v>
+      </c>
+      <c r="B97" s="28" t="s">
+        <v>315</v>
+      </c>
+      <c r="C97" s="28" t="s">
+        <v>351</v>
+      </c>
       <c r="D97" s="29" t="s">
-        <v>146</v>
+        <v>426</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D98" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D99" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D100" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D101" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B102" s="32" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D102" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D103" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B104" s="34" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C105" s="26" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D105" s="27" t="s">
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modif and commit round 16
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="253" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA247424-ECCB-4175-8CF7-412282A3F78A}"/>
+  <xr:revisionPtr revIDLastSave="258" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73656A77-D2C7-45C1-9DBE-0434E9B8CEEB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="426">
   <si>
     <t>Match</t>
   </si>
@@ -479,9 +479,6 @@
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>R16 Match 1 Winner vs R16 Match 2 Winner</t>
-  </si>
-  <si>
     <t>R16 Match 5 Winner vs R16 Match 6 Winner</t>
   </si>
   <si>
@@ -1106,12 +1103,6 @@
     <t>Panama</t>
   </si>
   <si>
-    <t>R16 Match 1 Winner</t>
-  </si>
-  <si>
-    <t>R16 Match 2 Winner</t>
-  </si>
-  <si>
     <t>R16 Match 5 Winner</t>
   </si>
   <si>
@@ -1317,6 +1308,12 @@
   </si>
   <si>
     <t>CHE COL</t>
+  </si>
+  <si>
+    <t>France vs Morocco</t>
+  </si>
+  <si>
+    <t>FRA MAR</t>
   </si>
 </sst>
 </file>
@@ -1957,22 +1954,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>308</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1980,22 +1977,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2003,22 +2000,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2026,22 +2023,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2049,22 +2046,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>309</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>310</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2072,22 +2069,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2095,22 +2092,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2118,22 +2115,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2141,22 +2138,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>315</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2164,22 +2161,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>315</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>316</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2187,22 +2184,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>313</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>314</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2210,22 +2207,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2233,22 +2230,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2256,22 +2253,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2279,22 +2276,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>318</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>319</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2302,22 +2299,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>319</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>320</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2325,22 +2322,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>317</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>318</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2348,22 +2345,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2371,22 +2368,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2394,22 +2391,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2417,22 +2414,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>322</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>323</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2440,22 +2437,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>323</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>324</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2463,22 +2460,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>321</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>322</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2486,22 +2483,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2509,22 +2506,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2532,22 +2529,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>325</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>326</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2555,22 +2552,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2578,22 +2575,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2601,22 +2598,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2624,22 +2621,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2647,22 +2644,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2670,22 +2667,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2693,22 +2690,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>329</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>330</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2716,22 +2713,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>328</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>329</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2739,22 +2736,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>330</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>331</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2762,22 +2759,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2785,22 +2782,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2808,22 +2805,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2831,22 +2828,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>333</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>334</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2854,22 +2851,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>331</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>332</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>333</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2877,22 +2874,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>334</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>335</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2900,22 +2897,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2923,22 +2920,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2946,22 +2943,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2969,22 +2966,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>337</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>338</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2992,22 +2989,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>336</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>337</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3015,22 +3012,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>338</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>339</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3038,22 +3035,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3061,22 +3058,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3084,22 +3081,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3107,22 +3104,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>341</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>342</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3130,22 +3127,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>340</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>341</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3153,22 +3150,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>342</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>343</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3176,22 +3173,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3199,22 +3196,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3222,22 +3219,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3245,22 +3242,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>344</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>345</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>346</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3268,22 +3265,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>343</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>344</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>345</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3291,22 +3288,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>346</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>347</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3314,22 +3311,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3337,22 +3334,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3360,22 +3357,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>347</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>348</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>349</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3383,22 +3380,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>349</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>350</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>351</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3406,22 +3403,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3429,22 +3426,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3452,22 +3449,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3475,22 +3472,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>348</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>349</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>350</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3498,22 +3495,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>351</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>352</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>353</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3521,22 +3518,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>353</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>354</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>355</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3544,22 +3541,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3567,22 +3564,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3590,22 +3587,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3613,758 +3610,758 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>352</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>353</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>354</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B74" s="26" t="s">
+        <v>311</v>
+      </c>
+      <c r="C74" s="26" t="s">
         <v>312</v>
       </c>
-      <c r="C74" s="26" t="s">
-        <v>313</v>
-      </c>
       <c r="D74" s="27" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="E74" s="48" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
+        <v>378</v>
+      </c>
+      <c r="B76" s="26" t="s">
+        <v>327</v>
+      </c>
+      <c r="C76" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="D76" s="27" t="s">
         <v>381</v>
       </c>
-      <c r="B76" s="26" t="s">
-        <v>328</v>
-      </c>
-      <c r="C76" s="26" t="s">
-        <v>320</v>
-      </c>
-      <c r="D76" s="27" t="s">
-        <v>384</v>
-      </c>
       <c r="E76" s="48" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
+        <v>379</v>
+      </c>
+      <c r="B77" s="26" t="s">
+        <v>316</v>
+      </c>
+      <c r="C77" s="26" t="s">
+        <v>330</v>
+      </c>
+      <c r="D77" s="27" t="s">
         <v>382</v>
       </c>
-      <c r="B77" s="26" t="s">
-        <v>317</v>
-      </c>
-      <c r="C77" s="26" t="s">
-        <v>331</v>
-      </c>
-      <c r="D77" s="27" t="s">
-        <v>385</v>
-      </c>
       <c r="E77" s="48" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C79" s="26" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D79" s="27" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="E79" s="48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
+        <v>380</v>
+      </c>
+      <c r="B82" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C82" s="26" t="s">
+        <v>315</v>
+      </c>
+      <c r="D82" s="27" t="s">
         <v>383</v>
       </c>
-      <c r="B82" s="26" t="s">
-        <v>321</v>
-      </c>
-      <c r="C82" s="26" t="s">
-        <v>316</v>
-      </c>
-      <c r="D82" s="27" t="s">
-        <v>386</v>
-      </c>
       <c r="E82" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="E91" s="49" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="E94" s="49" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D95" s="29" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E95" s="49" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
-        <v>147</v>
+        <v>424</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>356</v>
+        <v>339</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>357</v>
+        <v>319</v>
       </c>
       <c r="D98" s="31" t="s">
-        <v>146</v>
+        <v>425</v>
       </c>
       <c r="E98" s="50" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D99" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E99" s="50" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="D100" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E100" s="50" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D101" s="31" t="s">
         <v>146</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B102" s="32" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D102" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D103" s="33" t="s">
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B104" s="34" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B105" s="26" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C105" s="26" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D105" s="27" t="s">
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit end of round of 16, quarterfinal done
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="272" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{264FB18E-E3F3-416A-8484-9221B1ED900D}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C0FD870-C30A-4E54-8329-73D690030BC7}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="415">
   <si>
     <t>Match</t>
   </si>
@@ -479,9 +479,6 @@
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>R16 Match 7 Winner vs R16 Match 8 Winner</t>
-  </si>
-  <si>
     <t>QF Match 1 Winner vs QF Match 2 Winner</t>
   </si>
   <si>
@@ -1278,6 +1275,12 @@
   </si>
   <si>
     <t>ESP BEL</t>
+  </si>
+  <si>
+    <t>ARG CHE</t>
+  </si>
+  <si>
+    <t>Argentina vs Switzerland</t>
   </si>
 </sst>
 </file>
@@ -1918,22 +1921,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1941,22 +1944,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1964,22 +1967,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>308</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1987,22 +1990,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>309</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2010,22 +2013,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>306</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>307</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2033,22 +2036,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2056,22 +2059,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2079,22 +2082,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2102,22 +2105,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>311</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>312</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2125,22 +2128,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>312</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>313</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2148,22 +2151,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>310</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>311</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2171,22 +2174,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2194,22 +2197,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2217,22 +2220,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2240,22 +2243,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>315</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>316</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2263,22 +2266,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>316</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>317</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2286,22 +2289,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>314</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>315</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2309,22 +2312,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2332,22 +2335,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2355,22 +2358,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2378,22 +2381,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>319</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>320</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2401,22 +2404,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>320</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>321</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2424,22 +2427,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>318</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>319</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2447,22 +2450,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2470,22 +2473,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2493,22 +2496,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>322</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>323</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2516,22 +2519,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2539,22 +2542,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2562,22 +2565,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2585,22 +2588,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2608,22 +2611,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2631,22 +2634,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2654,22 +2657,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>326</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>327</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2677,22 +2680,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>325</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>326</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2700,22 +2703,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>327</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>328</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2723,22 +2726,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2746,22 +2749,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2769,22 +2772,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2792,22 +2795,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>330</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>331</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2815,22 +2818,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>329</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>330</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2838,22 +2841,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>331</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>332</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2861,22 +2864,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2884,22 +2887,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2907,22 +2910,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2930,22 +2933,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>334</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>335</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2953,22 +2956,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>333</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>334</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2976,22 +2979,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>334</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>335</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>336</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2999,22 +3002,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3022,22 +3025,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3045,22 +3048,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3068,22 +3071,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>338</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>339</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3091,22 +3094,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>337</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>338</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3114,22 +3117,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>339</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>340</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3137,22 +3140,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3160,22 +3163,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3183,22 +3186,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3206,22 +3209,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>341</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>342</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>343</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3229,22 +3232,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>340</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>341</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>342</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3252,22 +3255,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>342</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>343</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>344</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3275,22 +3278,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3298,22 +3301,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3321,22 +3324,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>344</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>345</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>346</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3344,22 +3347,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>346</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>347</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>348</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3367,22 +3370,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3390,22 +3393,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3413,22 +3416,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3436,22 +3439,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>345</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>346</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>347</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3459,22 +3462,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>348</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>349</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>350</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3482,22 +3485,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>350</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>351</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>352</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3505,22 +3508,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3528,22 +3531,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3551,22 +3554,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3574,667 +3577,671 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>349</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>350</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>351</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
+        <v>359</v>
+      </c>
+      <c r="B74" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="C74" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="D74" s="27" t="s">
         <v>360</v>
       </c>
-      <c r="B74" s="26" t="s">
-        <v>309</v>
-      </c>
-      <c r="C74" s="26" t="s">
-        <v>310</v>
-      </c>
-      <c r="D74" s="27" t="s">
-        <v>361</v>
-      </c>
       <c r="E74" s="48" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C79" s="26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D79" s="27" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E79" s="48" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
+        <v>391</v>
+      </c>
+      <c r="B91" s="28" t="s">
+        <v>309</v>
+      </c>
+      <c r="C91" s="28" t="s">
+        <v>316</v>
+      </c>
+      <c r="D91" s="29" t="s">
         <v>392</v>
       </c>
-      <c r="B91" s="28" t="s">
-        <v>310</v>
-      </c>
-      <c r="C91" s="28" t="s">
-        <v>317</v>
-      </c>
-      <c r="D91" s="29" t="s">
-        <v>393</v>
-      </c>
       <c r="E91" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
+        <v>399</v>
+      </c>
+      <c r="B94" s="28" t="s">
+        <v>344</v>
+      </c>
+      <c r="C94" s="28" t="s">
+        <v>332</v>
+      </c>
+      <c r="D94" s="29" t="s">
         <v>400</v>
       </c>
-      <c r="B94" s="28" t="s">
-        <v>345</v>
-      </c>
-      <c r="C94" s="28" t="s">
-        <v>333</v>
-      </c>
-      <c r="D94" s="29" t="s">
-        <v>401</v>
-      </c>
       <c r="E94" s="49" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
+        <v>397</v>
+      </c>
+      <c r="B95" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C95" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="D95" s="29" t="s">
         <v>398</v>
       </c>
-      <c r="B95" s="28" t="s">
-        <v>318</v>
-      </c>
-      <c r="C95" s="28" t="s">
-        <v>329</v>
-      </c>
-      <c r="D95" s="29" t="s">
-        <v>399</v>
-      </c>
       <c r="E95" s="49" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
+        <v>407</v>
+      </c>
+      <c r="B98" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="C98" s="30" t="s">
+        <v>316</v>
+      </c>
+      <c r="D98" s="31" t="s">
         <v>408</v>
       </c>
-      <c r="B98" s="30" t="s">
-        <v>337</v>
-      </c>
-      <c r="C98" s="30" t="s">
-        <v>317</v>
-      </c>
-      <c r="D98" s="31" t="s">
-        <v>409</v>
-      </c>
       <c r="E98" s="50" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
+        <v>411</v>
+      </c>
+      <c r="B99" s="31" t="s">
+        <v>332</v>
+      </c>
+      <c r="C99" s="30" t="s">
+        <v>328</v>
+      </c>
+      <c r="D99" s="31" t="s">
         <v>412</v>
       </c>
-      <c r="B99" s="31" t="s">
-        <v>333</v>
-      </c>
-      <c r="C99" s="30" t="s">
-        <v>329</v>
-      </c>
-      <c r="D99" s="31" t="s">
-        <v>413</v>
-      </c>
       <c r="E99" s="50" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
+        <v>409</v>
+      </c>
+      <c r="B100" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="C100" s="30" t="s">
+        <v>348</v>
+      </c>
+      <c r="D100" s="31" t="s">
         <v>410</v>
       </c>
-      <c r="B100" s="31" t="s">
-        <v>339</v>
-      </c>
-      <c r="C100" s="30" t="s">
-        <v>349</v>
-      </c>
-      <c r="D100" s="31" t="s">
-        <v>411</v>
-      </c>
       <c r="E100" s="50" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B101" s="30"/>
-      <c r="C101" s="30"/>
+        <v>414</v>
+      </c>
+      <c r="B101" s="30" t="s">
+        <v>340</v>
+      </c>
+      <c r="C101" s="30" t="s">
+        <v>311</v>
+      </c>
       <c r="D101" s="31" t="s">
-        <v>146</v>
+        <v>413</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B102" s="32"/>
       <c r="C102" s="32"/>
@@ -4242,18 +4249,18 @@
         <v>146</v>
       </c>
       <c r="E102" s="51" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B103" s="32"/>
       <c r="C103" s="32"/>
@@ -4261,18 +4268,18 @@
         <v>146</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B104" s="34"/>
       <c r="C104" s="34"/>
@@ -4280,18 +4287,18 @@
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B105" s="26"/>
       <c r="C105" s="26"/>
@@ -4299,13 +4306,13 @@
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit end of quarters
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="284" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D2A67E1-9E04-4C92-BD83-17C3849FCFA4}"/>
+  <xr:revisionPtr revIDLastSave="288" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24595577-9245-4F8E-91E5-068D2750365F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="416">
   <si>
     <t>Match</t>
   </si>
@@ -479,9 +479,6 @@
     <t>TBD TBD</t>
   </si>
   <si>
-    <t>QF Match 3 Winner vs QF Match 4 Winner</t>
-  </si>
-  <si>
     <t>SF Match 1 Loser vs SF Match 2 Loser</t>
   </si>
   <si>
@@ -1281,6 +1278,12 @@
   </si>
   <si>
     <t>FRA ESP</t>
+  </si>
+  <si>
+    <t>England vs Argentina</t>
+  </si>
+  <si>
+    <t>ENG ARG</t>
   </si>
 </sst>
 </file>
@@ -1921,22 +1924,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>302</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1944,22 +1947,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1967,22 +1970,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>304</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>305</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -1990,22 +1993,22 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>305</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>306</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2013,22 +2016,22 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>304</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2036,22 +2039,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2059,22 +2062,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2082,22 +2085,22 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2105,22 +2108,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>308</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>309</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2128,22 +2131,22 @@
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>309</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>310</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2151,22 +2154,22 @@
         <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>307</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2174,22 +2177,22 @@
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2197,22 +2200,22 @@
         <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2220,22 +2223,22 @@
         <v>26</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2243,22 +2246,22 @@
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>312</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>313</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2266,22 +2269,22 @@
         <v>30</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>313</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>314</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2289,22 +2292,22 @@
         <v>32</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>311</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>312</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2312,22 +2315,22 @@
         <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2335,22 +2338,22 @@
         <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2358,22 +2361,22 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="39" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2381,22 +2384,22 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>316</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>317</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>41</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2404,22 +2407,22 @@
         <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>317</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>318</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2427,22 +2430,22 @@
         <v>44</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>315</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>316</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2450,22 +2453,22 @@
         <v>46</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2473,22 +2476,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2496,22 +2499,22 @@
         <v>50</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>319</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>320</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2519,22 +2522,22 @@
         <v>52</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2542,22 +2545,22 @@
         <v>54</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>55</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2565,22 +2568,22 @@
         <v>56</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2588,22 +2591,22 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2611,22 +2614,22 @@
         <v>60</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2634,22 +2637,22 @@
         <v>62</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>63</v>
       </c>
       <c r="E32" s="41" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2657,22 +2660,22 @@
         <v>64</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>323</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>324</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>65</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2680,22 +2683,22 @@
         <v>66</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>322</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>323</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>67</v>
       </c>
       <c r="E34" s="41" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2703,22 +2706,22 @@
         <v>68</v>
       </c>
       <c r="B35" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>324</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>325</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>69</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2726,22 +2729,22 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>71</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2749,22 +2752,22 @@
         <v>72</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E37" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2772,22 +2775,22 @@
         <v>74</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E38" s="42" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2795,22 +2798,22 @@
         <v>76</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>326</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>327</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>328</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E39" s="42" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2818,22 +2821,22 @@
         <v>78</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>325</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>326</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>327</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>79</v>
       </c>
       <c r="E40" s="42" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2841,22 +2844,22 @@
         <v>80</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>327</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>328</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>329</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F41" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2864,22 +2867,22 @@
         <v>82</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="42" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2887,22 +2890,22 @@
         <v>84</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>85</v>
       </c>
       <c r="E43" s="42" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F43" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2910,22 +2913,22 @@
         <v>86</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2933,22 +2936,22 @@
         <v>88</v>
       </c>
       <c r="B45" s="16" t="s">
+        <v>330</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>331</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>332</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E45" s="43" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F45" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2956,22 +2959,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>330</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>331</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E46" s="43" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -2979,22 +2982,22 @@
         <v>92</v>
       </c>
       <c r="B47" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>332</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>333</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="43" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F47" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3002,22 +3005,22 @@
         <v>94</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E48" s="43" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3025,22 +3028,22 @@
         <v>96</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>97</v>
       </c>
       <c r="E49" s="43" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3048,22 +3051,22 @@
         <v>98</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>99</v>
       </c>
       <c r="E50" s="44" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3071,22 +3074,22 @@
         <v>100</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>335</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>336</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3094,22 +3097,22 @@
         <v>102</v>
       </c>
       <c r="B52" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="C52" s="18" t="s">
         <v>334</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>335</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>103</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3117,22 +3120,22 @@
         <v>104</v>
       </c>
       <c r="B53" s="18" t="s">
+        <v>335</v>
+      </c>
+      <c r="C53" s="18" t="s">
         <v>336</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>337</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>105</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F53" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3140,22 +3143,22 @@
         <v>106</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>107</v>
       </c>
       <c r="E54" s="44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3163,22 +3166,22 @@
         <v>108</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>109</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3186,22 +3189,22 @@
         <v>110</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>111</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F56" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3209,22 +3212,22 @@
         <v>112</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>338</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>339</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>340</v>
       </c>
       <c r="D57" s="21" t="s">
         <v>113</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F57" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3232,22 +3235,22 @@
         <v>114</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>337</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>338</v>
-      </c>
-      <c r="C58" s="20" t="s">
-        <v>339</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>115</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3255,22 +3258,22 @@
         <v>116</v>
       </c>
       <c r="B59" s="20" t="s">
+        <v>339</v>
+      </c>
+      <c r="C59" s="20" t="s">
         <v>340</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>341</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3278,22 +3281,22 @@
         <v>118</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>119</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3301,22 +3304,22 @@
         <v>120</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D61" s="21" t="s">
         <v>121</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F61" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3324,22 +3327,22 @@
         <v>122</v>
       </c>
       <c r="B62" s="22" t="s">
+        <v>341</v>
+      </c>
+      <c r="C62" s="22" t="s">
         <v>342</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>343</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>123</v>
       </c>
       <c r="E62" s="46" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3347,22 +3350,22 @@
         <v>124</v>
       </c>
       <c r="B63" s="22" t="s">
+        <v>343</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>344</v>
-      </c>
-      <c r="C63" s="22" t="s">
-        <v>345</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>125</v>
       </c>
       <c r="E63" s="46" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3370,22 +3373,22 @@
         <v>126</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D64" s="23" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="46" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F64" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3393,22 +3396,22 @@
         <v>128</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D65" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E65" s="46" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G65" s="23" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3416,22 +3419,22 @@
         <v>130</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>131</v>
       </c>
       <c r="E66" s="46" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3439,22 +3442,22 @@
         <v>132</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="C67" s="22" t="s">
         <v>343</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>344</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>133</v>
       </c>
       <c r="E67" s="46" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3462,22 +3465,22 @@
         <v>134</v>
       </c>
       <c r="B68" s="24" t="s">
+        <v>345</v>
+      </c>
+      <c r="C68" s="24" t="s">
         <v>346</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>347</v>
       </c>
       <c r="D68" s="25" t="s">
         <v>135</v>
       </c>
       <c r="E68" s="47" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3485,22 +3488,22 @@
         <v>136</v>
       </c>
       <c r="B69" s="24" t="s">
+        <v>347</v>
+      </c>
+      <c r="C69" s="24" t="s">
         <v>348</v>
-      </c>
-      <c r="C69" s="24" t="s">
-        <v>349</v>
       </c>
       <c r="D69" s="25" t="s">
         <v>137</v>
       </c>
       <c r="E69" s="47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3508,22 +3511,22 @@
         <v>138</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C70" s="24" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D70" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3531,22 +3534,22 @@
         <v>140</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D71" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="47" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3554,22 +3557,22 @@
         <v>142</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D72" s="25" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="47" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -3577,713 +3580,717 @@
         <v>144</v>
       </c>
       <c r="B73" s="24" t="s">
+        <v>346</v>
+      </c>
+      <c r="C73" s="24" t="s">
         <v>347</v>
-      </c>
-      <c r="C73" s="24" t="s">
-        <v>348</v>
       </c>
       <c r="D73" s="25" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="47" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
+        <v>356</v>
+      </c>
+      <c r="B74" s="26" t="s">
+        <v>305</v>
+      </c>
+      <c r="C74" s="26" t="s">
+        <v>306</v>
+      </c>
+      <c r="D74" s="27" t="s">
         <v>357</v>
       </c>
-      <c r="B74" s="26" t="s">
-        <v>306</v>
-      </c>
-      <c r="C74" s="26" t="s">
-        <v>307</v>
-      </c>
-      <c r="D74" s="27" t="s">
-        <v>358</v>
-      </c>
       <c r="E74" s="48" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F74" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B75" s="26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E75" s="48" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F75" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G75" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B76" s="26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C76" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E76" s="48" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F76" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G76" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B77" s="26" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E77" s="48" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F77" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="26" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B78" s="26" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C78" s="26" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E78" s="48" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F78" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="26" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C79" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D79" s="27" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E79" s="48" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B80" s="26" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G80" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B81" s="26" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C81" s="26" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E81" s="48" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F81" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G81" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="26" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B82" s="26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E82" s="48" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F82" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="26" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C83" s="26" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E83" s="48" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F83" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="26" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E84" s="48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F84" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C85" s="26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D85" s="27" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E85" s="48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F85" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G85" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B86" s="26" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C86" s="26" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E86" s="48" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F86" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G86" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="26" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B87" s="26" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C87" s="26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D87" s="27" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E87" s="48" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F87" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="26" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B88" s="26" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C88" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D88" s="27" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E88" s="48" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F88" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="26" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B89" s="26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C89" s="26" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D89" s="27" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E89" s="48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="28" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E90" s="49" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F90" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G90" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
+        <v>388</v>
+      </c>
+      <c r="B91" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="C91" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="D91" s="29" t="s">
         <v>389</v>
       </c>
-      <c r="B91" s="28" t="s">
-        <v>307</v>
-      </c>
-      <c r="C91" s="28" t="s">
-        <v>314</v>
-      </c>
-      <c r="D91" s="29" t="s">
-        <v>390</v>
-      </c>
       <c r="E91" s="49" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F91" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G91" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="28" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E92" s="49" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F92" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G92" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F93" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G93" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="28" t="s">
+        <v>396</v>
+      </c>
+      <c r="B94" s="28" t="s">
+        <v>341</v>
+      </c>
+      <c r="C94" s="28" t="s">
+        <v>329</v>
+      </c>
+      <c r="D94" s="29" t="s">
         <v>397</v>
       </c>
-      <c r="B94" s="28" t="s">
-        <v>342</v>
-      </c>
-      <c r="C94" s="28" t="s">
-        <v>330</v>
-      </c>
-      <c r="D94" s="29" t="s">
-        <v>398</v>
-      </c>
       <c r="E94" s="49" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F94" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G94" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
+        <v>394</v>
+      </c>
+      <c r="B95" s="28" t="s">
+        <v>314</v>
+      </c>
+      <c r="C95" s="28" t="s">
+        <v>325</v>
+      </c>
+      <c r="D95" s="29" t="s">
         <v>395</v>
       </c>
-      <c r="B95" s="28" t="s">
-        <v>315</v>
-      </c>
-      <c r="C95" s="28" t="s">
-        <v>326</v>
-      </c>
-      <c r="D95" s="29" t="s">
-        <v>396</v>
-      </c>
       <c r="E95" s="49" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F95" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G95" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="28" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E96" s="49" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F96" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G96" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E97" s="49" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F97" s="49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="30" t="s">
+        <v>404</v>
+      </c>
+      <c r="B98" s="30" t="s">
+        <v>333</v>
+      </c>
+      <c r="C98" s="30" t="s">
+        <v>313</v>
+      </c>
+      <c r="D98" s="31" t="s">
         <v>405</v>
       </c>
-      <c r="B98" s="30" t="s">
-        <v>334</v>
-      </c>
-      <c r="C98" s="30" t="s">
-        <v>314</v>
-      </c>
-      <c r="D98" s="31" t="s">
-        <v>406</v>
-      </c>
       <c r="E98" s="50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F98" s="50" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G98" s="31" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="30" t="s">
+        <v>408</v>
+      </c>
+      <c r="B99" s="31" t="s">
+        <v>329</v>
+      </c>
+      <c r="C99" s="30" t="s">
+        <v>325</v>
+      </c>
+      <c r="D99" s="31" t="s">
         <v>409</v>
       </c>
-      <c r="B99" s="31" t="s">
-        <v>330</v>
-      </c>
-      <c r="C99" s="30" t="s">
-        <v>326</v>
-      </c>
-      <c r="D99" s="31" t="s">
-        <v>410</v>
-      </c>
       <c r="E99" s="50" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F99" s="50" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="30" t="s">
+        <v>406</v>
+      </c>
+      <c r="B100" s="31" t="s">
+        <v>335</v>
+      </c>
+      <c r="C100" s="30" t="s">
+        <v>345</v>
+      </c>
+      <c r="D100" s="31" t="s">
         <v>407</v>
       </c>
-      <c r="B100" s="31" t="s">
-        <v>336</v>
-      </c>
-      <c r="C100" s="30" t="s">
-        <v>346</v>
-      </c>
-      <c r="D100" s="31" t="s">
-        <v>408</v>
-      </c>
       <c r="E100" s="50" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F100" s="50" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C101" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D101" s="31" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F101" s="50" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="32" t="s">
+        <v>412</v>
+      </c>
+      <c r="B102" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="C102" s="32" t="s">
+        <v>329</v>
+      </c>
+      <c r="D102" s="33" t="s">
         <v>413</v>
       </c>
-      <c r="B102" s="32" t="s">
-        <v>334</v>
-      </c>
-      <c r="C102" s="32" t="s">
-        <v>330</v>
-      </c>
-      <c r="D102" s="33" t="s">
-        <v>414</v>
-      </c>
       <c r="E102" s="51" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F102" s="51" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G102" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="B103" s="32"/>
-      <c r="C103" s="32"/>
+        <v>414</v>
+      </c>
+      <c r="B103" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="C103" s="32" t="s">
+        <v>337</v>
+      </c>
       <c r="D103" s="33" t="s">
-        <v>146</v>
+        <v>415</v>
       </c>
       <c r="E103" s="51" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F103" s="51" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G103" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B104" s="34"/>
       <c r="C104" s="34"/>
@@ -4291,18 +4298,18 @@
         <v>146</v>
       </c>
       <c r="E104" s="52" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F104" s="52" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B105" s="26"/>
       <c r="C105" s="26"/>
@@ -4310,13 +4317,13 @@
         <v>146</v>
       </c>
       <c r="E105" s="48" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F105" s="48" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit 1st semi final
</commit_message>
<xml_diff>
--- a/gameschedule.xlsx
+++ b/gameschedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="288" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24595577-9245-4F8E-91E5-068D2750365F}"/>
+  <xr:revisionPtr revIDLastSave="290" documentId="13_ncr:1_{73E7B376-678B-4EB2-8E7E-E35B22D34C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BF447CD-D295-47BC-830F-9CD11D3F8760}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="416">
   <si>
     <t>Match</t>
   </si>
@@ -4292,7 +4292,9 @@
       <c r="A104" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="B104" s="34"/>
+      <c r="B104" s="34" t="s">
+        <v>333</v>
+      </c>
       <c r="C104" s="34"/>
       <c r="D104" s="35" t="s">
         <v>146</v>
@@ -4311,7 +4313,9 @@
       <c r="A105" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="B105" s="26"/>
+      <c r="B105" s="26" t="s">
+        <v>329</v>
+      </c>
       <c r="C105" s="26"/>
       <c r="D105" s="27" t="s">
         <v>146</v>

</xml_diff>